<commit_message>
Govern Hurricane wind proxy range completion
</commit_message>
<xml_diff>
--- a/docs/cells/tropical_cyclone_wind_wind/proposed/damage_curve_records_tropical_cyclone_wind_wind__model_v1_1__docs_r1.xlsx
+++ b/docs/cells/tropical_cyclone_wind_wind/proposed/damage_curve_records_tropical_cyclone_wind_wind__model_v1_1__docs_r1.xlsx
@@ -710,7 +710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -778,14 +778,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TCWW11_CANONICAL_5MW_PROXY_V108P0</t>
+          <t>TCWW11_CANONICAL_5MW_PROXY_V100P0</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0006275236923301009</v>
+        <v>0</v>
       </c>
       <c r="D4" t="n">
         <v>0.63</v>
@@ -799,14 +799,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TCWW11_CANONICAL_5MW_PROXY_V160P0</t>
+          <t>TCWW11_CANONICAL_5MW_PROXY_V108P0</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>160</v>
+        <v>108</v>
       </c>
       <c r="C5" t="n">
-        <v>0.4235129655179889</v>
+        <v>0.0006275236923301009</v>
       </c>
       <c r="D5" t="n">
         <v>0.63</v>
@@ -820,14 +820,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TCWW11_CANONICAL_5MW_PROXY_V163P3</t>
+          <t>TCWW11_CANONICAL_5MW_PROXY_V160P0</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>163.3</v>
+        <v>160</v>
       </c>
       <c r="C6" t="n">
-        <v>0.5000000000000004</v>
+        <v>0.4235129655179889</v>
       </c>
       <c r="D6" t="n">
         <v>0.63</v>
@@ -841,14 +841,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TCWW11_CANONICAL_5MW_PROXY_V180P0</t>
+          <t>TCWW11_CANONICAL_5MW_PROXY_V163P3</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>180</v>
+        <v>163.3</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8548965899961662</v>
+        <v>0.5000000000000004</v>
       </c>
       <c r="D7" t="n">
         <v>0.63</v>
@@ -862,14 +862,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TCWW11_CANONICAL_5MW_PROXY_V200P0</t>
+          <t>TCWW11_CANONICAL_5MW_PROXY_V180P0</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="C8" t="n">
-        <v>0.9947744450209641</v>
+        <v>0.8548965899961662</v>
       </c>
       <c r="D8" t="n">
         <v>0.63</v>
@@ -883,19 +883,61 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TCWW11_CANONICAL_5MW_PROXY_V252P0</t>
+          <t>TCWW11_CANONICAL_5MW_PROXY_V200P0</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>252</v>
+        <v>200</v>
       </c>
       <c r="C9" t="n">
-        <v>0.9999999999999998</v>
+        <v>0.9947744450209641</v>
       </c>
       <c r="D9" t="n">
         <v>0.63</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>prohibited</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TCWW11_CANONICAL_5MW_PROXY_V252P0</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>252</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.9999999999999998</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>prohibited</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>TCWW11_CANONICAL_5MW_PROXY_V300P0</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>300</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>prohibited</t>
         </is>

</xml_diff>